<commit_message>
Pagina terminada solo falta actualizar datos
</commit_message>
<xml_diff>
--- a/Costeo_Velas.xlsx
+++ b/Costeo_Velas.xlsx
@@ -5,16 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iteso01-my.sharepoint.com/personal/ie722337_iteso_mx/Documents/Documentos/CASA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Velisima\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{367A4044-C7AB-489D-82AF-28455C81BDD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1389500B-FA8F-450A-8DAA-43555A30830E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D938DC7-20D8-4EB8-B797-A38FB8C04F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Costeo Velas" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
+    <sheet name="Fragancias" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>Molde</t>
   </si>
@@ -166,6 +166,18 @@
   </si>
   <si>
     <t>Peonía cempasuchil blanca</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>Costo_250ml</t>
+  </si>
+  <si>
+    <t>Costo_g</t>
   </si>
 </sst>
 </file>
@@ -217,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -230,6 +242,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -245,10 +260,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -674,7 +685,7 @@
         <v>35</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K28" si="6">J3-I3</f>
+        <f t="shared" ref="K3:K29" si="6">J3-I3</f>
         <v>31.09</v>
       </c>
       <c r="L3" t="s">
@@ -1785,8 +1796,13 @@
         <f>E29+G29+H29</f>
         <v>8.25</v>
       </c>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
+      <c r="J29" s="2">
+        <v>75</v>
+      </c>
+      <c r="K29" s="2">
+        <f t="shared" si="6"/>
+        <v>66.75</v>
+      </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1867,9 +1883,105 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB9274B-32B2-46BB-A88E-60A1CC0C5564}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="6.36328125" customWidth="1"/>
+    <col min="3" max="3" width="13.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>